<commit_message>
Last changes to paper green energy
</commit_message>
<xml_diff>
--- a/pasto_case/results/AHP_results/AHP_TOPSIS_results1.xlsx
+++ b/pasto_case/results/AHP_results/AHP_TOPSIS_results1.xlsx
@@ -478,249 +478,249 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>ICE</t>
+          <t>ICEV</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.07028192920485567</v>
+        <v>0.07030807929422099</v>
       </c>
       <c r="C2" t="n">
-        <v>0.03494452934456608</v>
+        <v>0.03488328220832244</v>
       </c>
       <c r="D2" t="n">
-        <v>0.00555135839304175</v>
+        <v>0.00507517465520403</v>
       </c>
       <c r="E2" t="n">
-        <v>0.0003072885977385833</v>
+        <v>0.0001196913259867757</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0002493572614815913</v>
+        <v>0.0004731435703355144</v>
       </c>
       <c r="G2" t="n">
-        <v>0.05506773823525951</v>
+        <v>0.04819289094843263</v>
       </c>
       <c r="H2" t="n">
-        <v>0.04325097357242033</v>
+        <v>0.04335609274534215</v>
       </c>
       <c r="I2" t="n">
-        <v>0.4399058203388902</v>
+        <v>0.4735835505325256</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>EVL1</t>
+          <t>EV-L1</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.02766252028443778</v>
+        <v>0.02742317169207324</v>
       </c>
       <c r="C3" t="n">
-        <v>0.031893758982</v>
+        <v>0.03168511399467544</v>
       </c>
       <c r="D3" t="n">
-        <v>0.01546873639797924</v>
+        <v>0.01856631376739243</v>
       </c>
       <c r="E3" t="n">
-        <v>0.01304855677303592</v>
+        <v>0.01174207655529854</v>
       </c>
       <c r="F3" t="n">
-        <v>0.004964087133505546</v>
+        <v>0.00680663015679641</v>
       </c>
       <c r="G3" t="n">
-        <v>0.06093460992513842</v>
+        <v>0.05420557764435638</v>
       </c>
       <c r="H3" t="n">
-        <v>0.01736460164356178</v>
+        <v>0.01916490074971436</v>
       </c>
       <c r="I3" t="n">
-        <v>0.2217723690400889</v>
+        <v>0.2612072480539139</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
         <is>
-          <t>EVL2</t>
+          <t>EV-L2</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.06734277776528666</v>
+        <v>0.06732284099777081</v>
       </c>
       <c r="C4" t="n">
-        <v>0.031893758982</v>
+        <v>0.03168511399467544</v>
       </c>
       <c r="D4" t="n">
-        <v>0.01546873639797924</v>
+        <v>0.01856631376739243</v>
       </c>
       <c r="E4" t="n">
-        <v>0.01304855677303592</v>
+        <v>0.01174207655529854</v>
       </c>
       <c r="F4" t="n">
-        <v>0.004964087133505546</v>
+        <v>0.00680663015679641</v>
       </c>
       <c r="G4" t="n">
-        <v>0.04354640682564953</v>
+        <v>0.03314897914312694</v>
       </c>
       <c r="H4" t="n">
-        <v>0.04331341852112405</v>
+        <v>0.04426372139179473</v>
       </c>
       <c r="I4" t="n">
-        <v>0.4986588258519096</v>
+        <v>0.571788880712499</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
-          <t>EVL3</t>
+          <t>EV-L3</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.0693202909441907</v>
+        <v>0.06940748589771241</v>
       </c>
       <c r="C5" t="n">
-        <v>0.031893758982</v>
+        <v>0.03168511399467544</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01497082324134114</v>
+        <v>0.01761814007627152</v>
       </c>
       <c r="E5" t="n">
-        <v>0.01304855677303592</v>
+        <v>0.01174207655529854</v>
       </c>
       <c r="F5" t="n">
-        <v>0.004964087133505546</v>
+        <v>0.00680663015679641</v>
       </c>
       <c r="G5" t="n">
-        <v>0.04394891385252109</v>
+        <v>0.03396270322216006</v>
       </c>
       <c r="H5" t="n">
-        <v>0.04502522824057298</v>
+        <v>0.04588345243193794</v>
       </c>
       <c r="I5" t="n">
-        <v>0.5060484673565367</v>
+        <v>0.5746482351725225</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>CNG</t>
+          <t>NGV</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>0.06341770424168119</v>
+        <v>0.06354770162368663</v>
       </c>
       <c r="C6" t="n">
-        <v>0.02758024402714348</v>
+        <v>0.02850868589969544</v>
       </c>
       <c r="D6" t="n">
-        <v>0.058779547817305</v>
+        <v>0.05141466748286392</v>
       </c>
       <c r="E6" t="n">
-        <v>0.003493911442838217</v>
+        <v>0.005921180415902573</v>
       </c>
       <c r="F6" t="n">
-        <v>0.0007166516589685644</v>
+        <v>0.00101357539818229</v>
       </c>
       <c r="G6" t="n">
-        <v>0.01502037132866975</v>
+        <v>0.01246395627444282</v>
       </c>
       <c r="H6" t="n">
-        <v>0.06420316392836417</v>
+        <v>0.05904472542510241</v>
       </c>
       <c r="I6" t="n">
-        <v>0.8104051872977209</v>
+        <v>0.8257000971320929</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>PHEVL1</t>
+          <t>PHEV-L1</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>0.06420857936254276</v>
+        <v>0.06417636246528356</v>
       </c>
       <c r="C7" t="n">
-        <v>0.03400851248965792</v>
+        <v>0.0339280925648797</v>
       </c>
       <c r="D7" t="n">
-        <v>0.008037079441821514</v>
+        <v>0.007703276941328855</v>
       </c>
       <c r="E7" t="n">
-        <v>0.008276932162597858</v>
+        <v>0.008836855146564388</v>
       </c>
       <c r="F7" t="n">
-        <v>0.006320846233754776</v>
+        <v>0.004304733194441361</v>
       </c>
       <c r="G7" t="n">
-        <v>0.05134893001874069</v>
+        <v>0.04433193848704422</v>
       </c>
       <c r="H7" t="n">
-        <v>0.03851615343709937</v>
+        <v>0.03844143527969934</v>
       </c>
       <c r="I7" t="n">
-        <v>0.4285997626211109</v>
+        <v>0.4644178862157752</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>PHEVL2</t>
+          <t>PHEV-L2</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>0.07019084042278959</v>
+        <v>0.07021065854932355</v>
       </c>
       <c r="C8" t="n">
-        <v>0.03400851248965792</v>
+        <v>0.0339280925648797</v>
       </c>
       <c r="D8" t="n">
-        <v>0.008037079441821514</v>
+        <v>0.007703276941328855</v>
       </c>
       <c r="E8" t="n">
-        <v>0.008276932162597858</v>
+        <v>0.008836855146564388</v>
       </c>
       <c r="F8" t="n">
-        <v>0.006320846233754776</v>
+        <v>0.004304733194441361</v>
       </c>
       <c r="G8" t="n">
-        <v>0.05097532978967835</v>
+        <v>0.04389012442478223</v>
       </c>
       <c r="H8" t="n">
-        <v>0.04423276675994824</v>
+        <v>0.04424608396130317</v>
       </c>
       <c r="I8" t="n">
-        <v>0.4645903905545702</v>
+        <v>0.5020193717374455</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>PHEVL3</t>
+          <t>PHEV-L3</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>0.07039485354471223</v>
+        <v>0.07042319525042535</v>
       </c>
       <c r="C9" t="n">
-        <v>0.03400851248965792</v>
+        <v>0.0339280925648797</v>
       </c>
       <c r="D9" t="n">
-        <v>0.008037079441821514</v>
+        <v>0.007703276941328855</v>
       </c>
       <c r="E9" t="n">
-        <v>0.008276932162597858</v>
+        <v>0.008836855146564388</v>
       </c>
       <c r="F9" t="n">
-        <v>0.006320846233754776</v>
+        <v>0.004304733194441361</v>
       </c>
       <c r="G9" t="n">
-        <v>0.05097492153807157</v>
+        <v>0.04388960982024732</v>
       </c>
       <c r="H9" t="n">
-        <v>0.04442895393003306</v>
+        <v>0.04445164721773714</v>
       </c>
       <c r="I9" t="n">
-        <v>0.4656933873182806</v>
+        <v>0.503181058411067</v>
       </c>
     </row>
   </sheetData>

</xml_diff>